<commit_message>
v2.0 tính theo đầu người
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EEC3C1A-38A9-491F-AE7D-2A7BAD8E79F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B2B57DA-D6F7-4568-AAF3-9F37316433E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kế hoạch dự án" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
cập nhật kế hoạch
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B2B57DA-D6F7-4568-AAF3-9F37316433E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F245A2D4-DACD-4B43-8E31-A644E5D92668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kế hoạch dự án" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="211">
   <si>
     <t>KẾ HOẠCH DỰ ÁN THEO AGILE/SCRUM</t>
   </si>
@@ -42,15 +42,6 @@
     <t>TÊN DỰ ÁN: Blue Moon</t>
   </si>
   <si>
-    <t>SCRUM MASTER: Trần Khánh Linh</t>
-  </si>
-  <si>
-    <t>NGÀY BẮT ĐẦU</t>
-  </si>
-  <si>
-    <t>NGÀY KẾT THÚC</t>
-  </si>
-  <si>
     <t>TIẾN ĐỘ TỔNG</t>
   </si>
   <si>
@@ -58,9 +49,6 @@
   </si>
   <si>
     <t>Phần mềm quản lý thu phí chung cư BlueMoon</t>
-  </si>
-  <si>
-    <t>0%</t>
   </si>
   <si>
     <t>v1.0: Quản lý thu phí, quản lý hộ khẩu/nhân khẩu, đăng nhập phân quyền.
@@ -129,9 +117,6 @@
     <t>NFR</t>
   </si>
   <si>
-    <t>Dev Team</t>
-  </si>
-  <si>
     <t>Cài đặt JDK 17+, MySQL 8+, IntelliJ IDEA, Git và Maven để phục vụ phát triển hệ thống Spring Boot.</t>
   </si>
   <si>
@@ -228,9 +213,6 @@
     <t>Cài đặt Audit Log (nhật ký thao tác)</t>
   </si>
   <si>
-    <t>Ghi log bằng @Slf4j format [AUDIT] thay vì bảng DB. Liên kết RL-023, NFR-003.</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Cài đặt Trạng thái thu phí theo căn hộ</t>
   </si>
   <si>
@@ -255,311 +237,448 @@
     <t>Hộp trắng + hộp đen. Liên kết RL-024.</t>
   </si>
   <si>
+    <t xml:space="preserve">    Cài đặt Quản lý người dùng (CRUD NguoiDung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Quản lý Loại khoản thu (LoaiKhoanThu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt trang Theo dõi thu phí tổng hợp</t>
+  </si>
+  <si>
+    <t>Sprint 3 — Thống kê, Báo cáo &amp; Hoàn thiện</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Thống kê (RL-011), xuất báo cáo (RL-012), tra cứu nợ (RL-010), đổi mật khẩu (RL-003), refactor &amp; kiểm thử tổng thể.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Thống kê các khoản đóng góp</t>
+  </si>
+  <si>
+    <t>Tổng tiền/đợt, số hộ nộp, chi tiết từng hộ. Liên kết RL-011.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Tra cứu nợ phí</t>
+  </si>
+  <si>
+    <t>Danh sách hộ nợ, số tiền, lần nộp cuối. Liên kết RL-010.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Quản lý phí gửi xe</t>
+  </si>
+  <si>
+    <t>Tạo loại khoản thu xe máy/ô tô, tính tự động. Liên kết RL-019, RL-014.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Import dữ liệu từ Excel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Xuất báo cáo (Excel/PDF)</t>
+  </si>
+  <si>
+    <t>Export báo cáo tổng thể. Liên kết RL-012.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Đổi mật khẩu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Refactor mã nguồn &amp; áp dụng Coding Convention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Kiểm thử tích hợp toàn bộ luồng nghiệp vụ</t>
+  </si>
+  <si>
+    <t>4 luồng: đăng nhập, tạo khoản thu, thu phí, thống kê.</t>
+  </si>
+  <si>
+    <t>CHÚ GIẢI TRẠNG THÁI</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Overdue</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>PRODUCT BACKLOG — BlueMoon Fee Management System</t>
+  </si>
+  <si>
+    <t>ƯU TIÊN</t>
+  </si>
+  <si>
+    <t>MÃ RL</t>
+  </si>
+  <si>
+    <t>USER STORY</t>
+  </si>
+  <si>
+    <t>SPRINT DỰ KIẾN</t>
+  </si>
+  <si>
+    <t>GHI CHÚ</t>
+  </si>
+  <si>
+    <t>RL-001</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn đăng nhập bằng tài khoản/mật khẩu.</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>RL-002</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn phân quyền kế toán / trưởng ban rõ ràng.</t>
+  </si>
+  <si>
+    <t>RL-004</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn tạo khoản thu mới (bắt buộc/tự nguyện).</t>
+  </si>
+  <si>
+    <t>RL-005</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn sửa/xóa khoản thu khi phát hiện sai sót.</t>
+  </si>
+  <si>
+    <t>RL-006</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn xem danh sách khoản thu, lọc theo loại/trạng thái.</t>
+  </si>
+  <si>
+    <t>RL-007</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn ghi nhận thanh toán của từng hộ theo mã căn hộ.</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>RL-008</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn tìm nhanh hộ gia đình và lọc theo trạng thái đóng phí.</t>
+  </si>
+  <si>
+    <t>RL-009</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn theo dõi trạng thái thu phí từng căn hộ.</t>
+  </si>
+  <si>
+    <t>RL-013</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn thêm/sửa/xóa thông tin hộ gia đình.</t>
+  </si>
+  <si>
+    <t>RL-014</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn quản lý nhân khẩu và ghi nhận biến động.</t>
+  </si>
+  <si>
+    <t>RL-010</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn biết cư dân nào còn nợ phí.</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>RL-011</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn thống kê tổng tiền thu mỗi đợt.</t>
+  </si>
+  <si>
+    <t>RL-012</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn xuất báo cáo ra Excel/PDF.</t>
+  </si>
+  <si>
+    <t>RL-003</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn đổi mật khẩu đăng nhập.</t>
+  </si>
+  <si>
+    <t>RL-015</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn tra cứu chi tiết hộ khẩu/nhân khẩu.</t>
+  </si>
+  <si>
+    <t>RL-021</t>
+  </si>
+  <si>
+    <t>Hệ thống phải xác thực người dùng trước khi cho phép truy cập.</t>
+  </si>
+  <si>
+    <t>RL-022</t>
+  </si>
+  <si>
+    <t>Hệ thống phải hỗ trợ phân quyền ít nhất 2 vai trò.</t>
+  </si>
+  <si>
+    <t>RL-024</t>
+  </si>
+  <si>
+    <t>Thời gian phản hồi mỗi thao tác &lt; 3 giây.</t>
+  </si>
+  <si>
+    <t>RL-019</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn quản lý phí gửi xe (xe máy/ô tô).</t>
+  </si>
+  <si>
+    <t>RL-023</t>
+  </si>
+  <si>
+    <t>Hệ thống phải ghi nhật ký mọi thao tác (ai, làm gì, lúc nào).</t>
+  </si>
+  <si>
+    <t>RL-018</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn import file Excel để cập nhật dữ liệu hàng loạt.</t>
+  </si>
+  <si>
+    <t>RL-016</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn hệ thống nhắc cư dân đóng phí.</t>
+  </si>
+  <si>
+    <t>v2.0</t>
+  </si>
+  <si>
+    <t>Có thể để v2.0</t>
+  </si>
+  <si>
+    <t>RL-020</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn thu hộ điện/nước/internet.</t>
+  </si>
+  <si>
+    <t>Sprint 4 — v2.0: Phí gửi xe &amp; Thu hộ</t>
+  </si>
+  <si>
+    <t>Hoàn thiện các tính năng v2.0: quản lý phí gửi xe (PER_XE), thu hộ điện/nước/internet (THU_HO), email nhắc nợ tự động (RL-016, RL-019, RL-020).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Quản lý phương tiện (PhuongTien CRUD)</t>
+  </si>
+  <si>
+    <t>Thêm/sửa/xóa xe máy/ô tô theo hộ, kiểm tra biển số trùng. Liên kết RL-019.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt tính phí PER_XE tự động theo số xe</t>
+  </si>
+  <si>
+    <t>Tự tính soTienYeuCau = số xe máy × giaXeMay + số ô tô × giaOto khi tạo ThanhToan. Liên kết RL-019.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt loại phí THU_HO (thu hộ điện/nước/internet)</t>
+  </si>
+  <si>
+    <t>Nhập số tiền riêng từng hộ qua form nhap-thu-ho. Liên kết RL-020.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Mẫu khoản thu định kỳ (MauKhoanThu)</t>
+  </si>
+  <si>
+    <t>Template tự động tạo KhoanThu mỗi tháng vào ngày 28, back-fill khi khởi động.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Email nhắc nợ tự động (EmailSchedulerService)</t>
+  </si>
+  <si>
+    <t>3 job: thứ Hai 8h (tất cả nợ), hằng ngày 8h (gần hạn 1–3 ngày), hằng ngày 9h (vừa quá hạn). Liên kết RL-016.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Lịch sử email &amp; Audit Log DB</t>
+  </si>
+  <si>
+    <t>Lưu mọi lần gửi email vào bảng lich_su_email; nâng Audit Log từ SLF4J lên bảng audit_log. Liên kết RL-023.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cài đặt Thùng rác (soft delete)</t>
+  </si>
+  <si>
+    <t>Xóa mềm HoGiaDinh và KhoanThu bằng deleted_at + @SQLRestriction; khôi phục/xóa vĩnh viễn tại /thung-rac.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Sprint Review &amp; Demo v2.0</t>
+  </si>
+  <si>
+    <t>Demo toàn bộ v2.0, chốt bàn giao sản phẩm hoàn chỉnh.</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Scrum Master: Trần Khánh Linh  |  Product Owner: Lê Quang Huy  |  Cập nhật lần cuối: 15/06/2026</t>
+  </si>
+  <si>
+    <t>RL-025</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn quản lý phương tiện của từng hộ gia đình.</t>
+  </si>
+  <si>
+    <t>PhuongTien CRUD, kiểm tra biển số trùng</t>
+  </si>
+  <si>
+    <t>RL-026</t>
+  </si>
+  <si>
+    <t>Hệ thống phải tự động tạo khoản thu định kỳ mỗi tháng theo mẫu.</t>
+  </si>
+  <si>
+    <t>MauKhoanThu scheduler ngày 28</t>
+  </si>
+  <si>
+    <t>RL-027</t>
+  </si>
+  <si>
+    <t>Hệ thống phải lưu lịch sử gửi email thông báo.</t>
+  </si>
+  <si>
+    <t>Bảng lich_su_email</t>
+  </si>
+  <si>
+    <t>CRUD tài khoản tại /nguoi-dung, tự bảo vệ (không tự xóa/đổi vai trò chính mình).</t>
+  </si>
+  <si>
+    <t>CRUD loại khoản thu tại /loai-khoan-thu, tách biệt khỏi module khoản thu.</t>
+  </si>
+  <si>
+    <t>Dùng Apache POI, validate dữ liệu trước khi lưu DB. Liên kết RL-018.</t>
+  </si>
+  <si>
+    <t>Đổi mật khẩu người dùng đang đăng nhập. Liên kết RL-003.</t>
+  </si>
+  <si>
+    <t>Bảng tất cả hộ vs trạng thái đóng phí tại /thanh-toan/theo-doi dùng paymentMap.</t>
+  </si>
+  <si>
+    <t>Ghi log theo format [AUDIT] Tạo|Sửa|Xóa entity bằng @Slf4j thay vì bảng DB riêng. Liên kết RL-023.</t>
+  </si>
+  <si>
+    <t>Tuân thủ Java Coding Convention, Javadocs.</t>
+  </si>
+  <si>
+    <t>RL-028</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn quản lý tài khoản người dùng hệ thống.</t>
+  </si>
+  <si>
+    <t>CRUD NguoiDung tại /nguoi-dung, tự bảo vệ tài khoản</t>
+  </si>
+  <si>
+    <t>RL-029</t>
+  </si>
+  <si>
+    <t>Là kế toán, tôi muốn quản lý danh mục loại khoản thu.</t>
+  </si>
+  <si>
+    <t>CRUD LoaiKhoanThu tại /loai-khoan-thu</t>
+  </si>
+  <si>
+    <t>RL-030</t>
+  </si>
+  <si>
+    <t>Hệ thống phải tự động áp phí bắt buộc cho mọi hộ khi tạo khoản thu.</t>
+  </si>
+  <si>
+    <t>autoApplyNeuBatBuoc, tạo ThanhToan CON_NO</t>
+  </si>
+  <si>
+    <t>RL-031</t>
+  </si>
+  <si>
+    <t>Là trưởng ban, tôi muốn theo dõi tổng hợp trạng thái thu phí của tất cả hộ.</t>
+  </si>
+  <si>
+    <t>Trang /thanh-toan/theo-doi, paymentMap</t>
+  </si>
+  <si>
+    <t>RL-032</t>
+  </si>
+  <si>
+    <t>Hệ thống phải hỗ trợ migration cơ sở dữ liệu theo phiên bản.</t>
+  </si>
+  <si>
+    <t>bluemoon_schema.sql + migration_v2..v6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Xây dựng hệ thống Database Migration theo phiên bản</t>
+  </si>
+  <si>
+    <t>Migration file đánh số phiên bản: bluemoon_schema.sql + migration_v2</t>
+  </si>
+  <si>
+    <t>TEAM LEADER: Lê Quang Huy
+PRODUCT OWNER: Lê Quang Huy
+SCRUM MASTER: Trần Khánh Linh</t>
+  </si>
+  <si>
+    <t>NGÀY KẾT THÚC: 12/06/2026</t>
+  </si>
+  <si>
+    <t>NGÀY BẮT ĐẦU: 27/3/2026</t>
+  </si>
+  <si>
+    <t>Lê Quang Huy</t>
+  </si>
+  <si>
+    <t>Trần Khánh Linh</t>
+  </si>
+  <si>
+    <t>Đặng Hải Đăng</t>
+  </si>
+  <si>
+    <t>Đoàn Văn Thắng</t>
+  </si>
+  <si>
     <t xml:space="preserve">    Sprint Review &amp; Retrospective Sprint 2</t>
   </si>
   <si>
-    <t>Demo, đánh giá tiến độ, cập nhật Backlog.</t>
-  </si>
-  <si>
-    <t>Bổ sung ngoài kế hoạch gốc — Sprint 1 &amp; 2</t>
-  </si>
-  <si>
-    <t>Các tính năng thực tế đã triển khai nhưng không có trong Product Backlog ban đầu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Quản lý người dùng (CRUD NguoiDung)</t>
-  </si>
-  <si>
-    <t>CRUD tài khoản tại /nguoi-dung, tự bảo vệ (không tự xóa/đổi vai trò chính mình). Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Quản lý Loại khoản thu (LoaiKhoanThu)</t>
-  </si>
-  <si>
-    <t>CRUD loại khoản thu tại /loai-khoan-thu, tách biệt khỏi module khoản thu. Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt trang Theo dõi thu phí tổng hợp</t>
-  </si>
-  <si>
-    <t>Bảng tất cả hộ vs trạng thái đóng phí tại /thanh-toan/theo-doi dùng paymentMap. Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt logic tự động áp phí bắt buộc (autoApplyNeuBatBuoc)</t>
-  </si>
-  <si>
-    <t>Tự tạo ThanhToan CON_NO cho mọi hộ khi có KhoanThu loại bắt buộc. Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Xây dựng hệ thống Database Migration theo phiên bản (v1–v6)</t>
-  </si>
-  <si>
-    <t>Migration file đánh số phiên bản: bluemoon_schema.sql + migration_v2..v6. Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Audit Log bằng SLF4J (format [AUDIT])</t>
-  </si>
-  <si>
-    <t>Ghi log theo format [AUDIT] Tạo|Sửa|Xóa entity bằng @Slf4j thay vì bảng DB riêng. Ngoài kế hoạch gốc.</t>
-  </si>
-  <si>
-    <t>Sprint 3 — Thống kê, Báo cáo &amp; Hoàn thiện</t>
-  </si>
-  <si>
-    <t>Not Started</t>
-  </si>
-  <si>
-    <t>Thống kê (RL-011), xuất báo cáo (RL-012), tra cứu nợ (RL-010), đổi mật khẩu (RL-003), refactor &amp; kiểm thử tổng thể.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Thống kê các khoản đóng góp</t>
-  </si>
-  <si>
-    <t>Tổng tiền/đợt, số hộ nộp, chi tiết từng hộ. Liên kết RL-011.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Tra cứu nợ phí</t>
-  </si>
-  <si>
-    <t>Danh sách hộ nợ, số tiền, lần nộp cuối. Liên kết RL-010.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Quản lý phí gửi xe</t>
-  </si>
-  <si>
-    <t>Tạo loại khoản thu xe máy/ô tô, tính tự động. Liên kết RL-019, RL-014.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Import dữ liệu từ Excel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dùng Apache POI, validate dữ liệu trước khi lưu DB. Liên kết RL-018. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Xuất báo cáo (Excel/PDF)</t>
-  </si>
-  <si>
-    <t>Export báo cáo tổng thể. Liên kết RL-012.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Cài đặt Đổi mật khẩu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Refactor mã nguồn &amp; áp dụng Coding Convention</t>
-  </si>
-  <si>
-    <t>Tuân thủ Java Coding Convention, Javadocs. Liên kết RL-027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Kiểm thử tích hợp toàn bộ luồng nghiệp vụ</t>
-  </si>
-  <si>
-    <t>4 luồng: đăng nhập, tạo khoản thu, thu phí, thống kê.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Hoàn thiện tài liệu dự án</t>
-  </si>
-  <si>
-    <t>SRS, thiết kế, test report, hướng dẫn cài đặt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Sprint Review &amp; Demo cuối — bàn giao v1.0</t>
-  </si>
-  <si>
-    <t>Demo toàn bộ sản phẩm, chốt bàn giao v1.0.</t>
-  </si>
-  <si>
-    <t>CHÚ GIẢI TRẠNG THÁI</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Overdue</t>
-  </si>
-  <si>
-    <t>Blocked</t>
-  </si>
-  <si>
-    <t>PRODUCT BACKLOG — BlueMoon Fee Management System</t>
-  </si>
-  <si>
-    <t>Scrum Master: Trần Khánh Linh  |  Product Owner: Lê Quang Huy  |  Cập nhật lần cuối: 31/03/2026</t>
-  </si>
-  <si>
-    <t>ƯU TIÊN</t>
-  </si>
-  <si>
-    <t>MÃ RL</t>
-  </si>
-  <si>
-    <t>USER STORY</t>
-  </si>
-  <si>
-    <t>SPRINT DỰ KIẾN</t>
-  </si>
-  <si>
-    <t>GHI CHÚ</t>
-  </si>
-  <si>
-    <t>RL-001</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn đăng nhập bằng tài khoản/mật khẩu.</t>
-  </si>
-  <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
-    <t>RL-002</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn phân quyền kế toán / trưởng ban rõ ràng.</t>
-  </si>
-  <si>
-    <t>RL-004</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn tạo khoản thu mới (bắt buộc/tự nguyện).</t>
-  </si>
-  <si>
-    <t>RL-005</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn sửa/xóa khoản thu khi phát hiện sai sót.</t>
-  </si>
-  <si>
-    <t>RL-006</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn xem danh sách khoản thu, lọc theo loại/trạng thái.</t>
-  </si>
-  <si>
-    <t>RL-007</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn ghi nhận thanh toán của từng hộ theo mã căn hộ.</t>
-  </si>
-  <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
-    <t>RL-008</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn tìm nhanh hộ gia đình và lọc theo trạng thái đóng phí.</t>
-  </si>
-  <si>
-    <t>RL-009</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn theo dõi trạng thái thu phí từng căn hộ.</t>
-  </si>
-  <si>
-    <t>RL-013</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn thêm/sửa/xóa thông tin hộ gia đình.</t>
-  </si>
-  <si>
-    <t>RL-014</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn quản lý nhân khẩu và ghi nhận biến động.</t>
-  </si>
-  <si>
-    <t>RL-010</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn biết cư dân nào còn nợ phí.</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
-    <t>RL-011</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn thống kê tổng tiền thu mỗi đợt.</t>
-  </si>
-  <si>
-    <t>RL-012</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn xuất báo cáo ra Excel/PDF.</t>
-  </si>
-  <si>
-    <t>RL-003</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn đổi mật khẩu đăng nhập.</t>
-  </si>
-  <si>
-    <t>RL-015</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn tra cứu chi tiết hộ khẩu/nhân khẩu.</t>
-  </si>
-  <si>
-    <t>RL-021</t>
-  </si>
-  <si>
-    <t>Hệ thống phải xác thực người dùng trước khi cho phép truy cập.</t>
-  </si>
-  <si>
-    <t>RL-022</t>
-  </si>
-  <si>
-    <t>Hệ thống phải hỗ trợ phân quyền ít nhất 2 vai trò.</t>
-  </si>
-  <si>
-    <t>RL-024</t>
-  </si>
-  <si>
-    <t>Thời gian phản hồi mỗi thao tác &lt; 3 giây.</t>
-  </si>
-  <si>
-    <t>RL-019</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn quản lý phí gửi xe (xe máy/ô tô).</t>
-  </si>
-  <si>
-    <t>RL-023</t>
-  </si>
-  <si>
-    <t>Hệ thống phải ghi nhật ký mọi thao tác (ai, làm gì, lúc nào).</t>
-  </si>
-  <si>
-    <t>RL-018</t>
-  </si>
-  <si>
-    <t>Là kế toán, tôi muốn import file Excel để cập nhật dữ liệu hàng loạt.</t>
-  </si>
-  <si>
-    <t>RL-016</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn hệ thống nhắc cư dân đóng phí.</t>
-  </si>
-  <si>
-    <t>v2.0</t>
-  </si>
-  <si>
-    <t>Có thể để v2.0</t>
-  </si>
-  <si>
-    <t>RL-020</t>
-  </si>
-  <si>
-    <t>Là trưởng ban, tôi muốn thu hộ điện/nước/internet.</t>
+    <t xml:space="preserve">    Sprint Review &amp; Retrospective Sprint 3</t>
+  </si>
+  <si>
+    <t>Demo toàn bộ v1.0, cập nhật Backlog. Lên kế hoạch cho v2.0</t>
+  </si>
+  <si>
+    <t>Ghi log bằng @Slf4j format [AUDIT] thay vì bảng DB cho các tính năng đã hoàn thành. Liên kết RL-023, NFR-003.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cập nhật Audit Log</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -665,36 +784,29 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color rgb="FF404040"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF404040"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1A5276"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF404040"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF7D4F00"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7D4F00"/>
-      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="163"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -781,17 +893,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -971,14 +1092,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1017,9 +1135,6 @@
     <xf numFmtId="1" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1083,9 +1198,6 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1137,43 +1249,64 @@
     <xf numFmtId="0" fontId="17" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1195,6 +1328,55 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1202,6 +1384,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF404040"/>
+      <color rgb="FFD9D9D9"/>
+      <color rgb="FFF2F2F2"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1409,16 +1598,38 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{2655DDF5-B1A8-41E5-BC89-AB17A4656B0B}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;058e744e-dad9-4a9c-a11e-46cc9bba6fd6&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K998"/>
+  <dimension ref="A1:K1006"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" customWidth="1"/>
     <col min="2" max="2" width="7.44140625" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="25.77734375" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="12.109375" customWidth="1"/>
     <col min="7" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
@@ -1428,1104 +1639,1276 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
-    </row>
-    <row r="2" spans="2:11" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+    </row>
+    <row r="2" spans="2:11" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="84" t="s">
+        <v>199</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G2" s="85"/>
+      <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="J2" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="K2" s="77"/>
+    </row>
+    <row r="3" spans="2:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="81"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="54">
+        <v>1</v>
+      </c>
+      <c r="J3" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="74" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" s="75"/>
-    </row>
-    <row r="3" spans="2:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="78" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J3" s="72" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="73"/>
+      <c r="K3" s="75"/>
     </row>
     <row r="4" spans="2:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="J5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="K5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="3" t="s">
+    </row>
+    <row r="6" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="3"/>
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="D6" s="5"/>
+      <c r="E6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="3" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="4"/>
-      <c r="C6" s="5" t="s">
+    <row r="7" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="7" t="s">
+      <c r="D7" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="8" t="s">
+      <c r="E7" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="10"/>
-      <c r="C7" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16" t="str">
+      <c r="F7" s="13"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15" t="str">
         <f>IF(AND(G7&lt;&gt;"",H7&lt;&gt;""),H7-G7,"")</f>
         <v/>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" s="18" t="s">
-        <v>27</v>
+      <c r="J7" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="19"/>
-      <c r="C8" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="25" t="str">
+      <c r="B8" s="17"/>
+      <c r="C8" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="91" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="23" t="str">
         <f>IF(AND(G8&lt;&gt;"",H8&lt;&gt;""),H8-G8,"")</f>
         <v/>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="9"/>
+      <c r="C9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="K8" s="26" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="10"/>
-      <c r="C9" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16" t="str">
+      <c r="F9" s="13"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="15" t="str">
         <f>IF(AND(G9&lt;&gt;"",H9&lt;&gt;""),H9-G9,"")</f>
         <v/>
       </c>
-      <c r="J9" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" s="18" t="s">
-        <v>33</v>
+      <c r="J9" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="19"/>
-      <c r="C10" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="25" t="str">
+      <c r="B10" s="17"/>
+      <c r="C10" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="91" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="21"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="23" t="str">
         <f>IF(AND(G10&lt;&gt;"",H10&lt;&gt;""),H10-G10,"")</f>
         <v/>
       </c>
-      <c r="J10" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="26" t="s">
-        <v>37</v>
+      <c r="J10" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="24" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="2:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4"/>
-      <c r="C12" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="8" t="s">
+      <c r="B12" s="3"/>
+      <c r="C12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="9" t="s">
-        <v>39</v>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="10"/>
-      <c r="C13" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16" t="str">
+      <c r="B13" s="9"/>
+      <c r="C13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="F13" s="13"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="15" t="str">
         <f t="shared" ref="I13:I19" si="0">IF(AND(G13&lt;&gt;"",H13&lt;&gt;""),H13-G13,"")</f>
         <v/>
       </c>
-      <c r="J13" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K13" s="18" t="s">
-        <v>41</v>
+      <c r="J13" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="19"/>
-      <c r="C14" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="23"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="25" t="str">
+      <c r="B14" s="17"/>
+      <c r="C14" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="F14" s="21"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="23" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J14" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K14" s="26" t="s">
-        <v>43</v>
+      <c r="J14" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K14" s="24" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="10"/>
-      <c r="C15" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" s="14"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="16" t="str">
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="F15" s="13"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J15" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K15" s="18" t="s">
-        <v>45</v>
+      <c r="J15" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="19"/>
-      <c r="C16" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E16" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" s="23"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="25" t="str">
+      <c r="B16" s="17"/>
+      <c r="C16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="F16" s="21"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J16" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K16" s="26" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="10"/>
-      <c r="C17" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="16" t="str">
+      <c r="J16" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="9"/>
+      <c r="C17" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="F17" s="13"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J17" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K17" s="18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="19"/>
-      <c r="C18" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" s="23"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="25" t="str">
+      <c r="J17" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="17"/>
+      <c r="C18" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="F18" s="21"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="23" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J18" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K18" s="26" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="10"/>
-      <c r="C19" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="16" t="str">
+      <c r="J18" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K18" s="24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="9"/>
+      <c r="C19" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="13"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J19" s="17" t="s">
+      <c r="J19" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="21" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="3"/>
+      <c r="C21" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="K19" s="18" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="4"/>
-      <c r="C21" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="10"/>
-      <c r="C22" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16" t="str">
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="9"/>
+      <c r="C22" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="15" t="str">
         <f t="shared" ref="I22:I32" si="1">IF(AND(G22&lt;&gt;"",H22&lt;&gt;""),H22-G22,"")</f>
         <v/>
       </c>
-      <c r="J22" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K22" s="18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="19"/>
-      <c r="C23" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="25" t="str">
+      <c r="J22" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="17"/>
+      <c r="C23" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J23" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K23" s="26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="10"/>
-      <c r="C24" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="16" t="str">
+      <c r="J23" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K23" s="24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="9"/>
+      <c r="C24" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" s="90" t="s">
+        <v>205</v>
+      </c>
+      <c r="F24" s="13"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J24" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="19"/>
-      <c r="C25" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F25" s="23"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="25" t="str">
+      <c r="J24" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="17"/>
+      <c r="C25" s="88" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="F25" s="21"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J25" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K25" s="26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="31"/>
-      <c r="C26" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="F26" s="35"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="37" t="str">
+      <c r="J25" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K25" s="100" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="29"/>
+      <c r="C26" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="F26" s="33"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="35" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J26" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K26" s="38" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="19"/>
-      <c r="C27" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F27" s="23"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="25" t="str">
+      <c r="J26" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K26" s="36" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="17"/>
+      <c r="C27" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="91" t="s">
+        <v>205</v>
+      </c>
+      <c r="F27" s="21"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J27" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K27" s="26" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="31"/>
-      <c r="C28" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="E28" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" s="35"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="37" t="str">
+      <c r="J27" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K27" s="24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="29"/>
+      <c r="C28" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="F28" s="33"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="35" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J28" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K28" s="38" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="19"/>
-      <c r="C29" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F29" s="23"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="25" t="str">
+      <c r="J28" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K28" s="36" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="17"/>
+      <c r="C29" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="F29" s="21"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J29" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="26" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="31"/>
-      <c r="C30" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="D30" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="E30" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="F30" s="35"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="37" t="str">
+      <c r="J29" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K29" s="24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="9"/>
+      <c r="C30" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F30" s="43"/>
+      <c r="G30" s="60"/>
+      <c r="H30" s="60"/>
+      <c r="I30" s="61" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J30" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="K30" s="38" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="64"/>
-      <c r="B31" s="64"/>
-      <c r="C31" s="65" t="s">
-        <v>74</v>
-      </c>
-      <c r="D31" s="66" t="s">
-        <v>25</v>
-      </c>
-      <c r="E31" s="67" t="s">
-        <v>30</v>
-      </c>
-      <c r="F31" s="64"/>
+      <c r="J30" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B31" s="17"/>
+      <c r="C31" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="F31" s="63"/>
       <c r="G31" s="64"/>
       <c r="H31" s="64"/>
-      <c r="I31" s="68" t="str">
+      <c r="I31" s="65" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J31" s="69" t="s">
-        <v>22</v>
-      </c>
-      <c r="K31" s="70" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C32" s="58" t="s">
-        <v>76</v>
-      </c>
-      <c r="D32" s="59" t="s">
-        <v>25</v>
-      </c>
-      <c r="E32" s="61" t="s">
+      <c r="J31" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" s="24" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="9"/>
+      <c r="C32" s="89" t="s">
+        <v>206</v>
+      </c>
+      <c r="D32" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="I32" s="71" t="str">
+      <c r="E32" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F32" s="13"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J32" s="62" t="s">
+      <c r="J32" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="34" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="3"/>
+      <c r="C34" s="56" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" s="57"/>
+      <c r="E34" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="K32" s="63" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C33" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="D33" s="59" t="s">
-        <v>25</v>
-      </c>
-      <c r="E33" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="I33" s="61" t="str">
-        <f t="shared" ref="I33:I37" si="2">IF(AND(G32&lt;&gt;"",H32&lt;&gt;""),H32-G32,"")</f>
+      <c r="F34" s="57"/>
+      <c r="G34" s="57"/>
+      <c r="H34" s="57"/>
+      <c r="I34" s="57"/>
+      <c r="J34" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B35" s="9"/>
+      <c r="C35" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F35" s="43"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="60"/>
+      <c r="I35" s="61" t="str">
+        <f t="shared" ref="I32:I36" si="2">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34,"")</f>
         <v/>
       </c>
-      <c r="J33" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K33" s="63" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="34" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C34" s="58" t="s">
-        <v>80</v>
-      </c>
-      <c r="D34" s="59" t="s">
-        <v>25</v>
-      </c>
-      <c r="E34" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="I34" s="61" t="str">
+      <c r="J35" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B36" s="17"/>
+      <c r="C36" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D36" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="F36" s="63"/>
+      <c r="G36" s="64"/>
+      <c r="H36" s="64"/>
+      <c r="I36" s="65" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="J34" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K34" s="63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="2:11" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C35" s="58" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="59" t="s">
-        <v>25</v>
-      </c>
-      <c r="E35" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="I35" s="61" t="str">
-        <f t="shared" si="2"/>
+      <c r="J36" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K36" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B37" s="9"/>
+      <c r="C37" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="F37" s="43"/>
+      <c r="G37" s="60"/>
+      <c r="H37" s="60"/>
+      <c r="I37" s="61"/>
+      <c r="J37" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B38" s="17"/>
+      <c r="C38" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D38" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="F38" s="63"/>
+      <c r="G38" s="64"/>
+      <c r="H38" s="64"/>
+      <c r="I38" s="65" t="str">
+        <f>IF(AND(G32&lt;&gt;"",H32&lt;&gt;""),H32-G32,"")</f>
         <v/>
       </c>
-      <c r="J35" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K35" s="63" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="36" spans="2:11" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C36" s="58" t="s">
-        <v>84</v>
-      </c>
-      <c r="D36" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="E36" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="I36" s="61" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J36" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K36" s="63" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="58" t="s">
-        <v>86</v>
-      </c>
-      <c r="D37" s="59" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="60" t="s">
-        <v>30</v>
-      </c>
-      <c r="I37" s="61" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="J37" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K37" s="63" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="38" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="4"/>
-      <c r="C38" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D38" s="6"/>
-      <c r="E38" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="K38" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="39" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="10"/>
-      <c r="C39" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="D39" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F39" s="14"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="15"/>
-      <c r="I39" s="16" t="str">
+      <c r="J38" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K38" s="24" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B39" s="9"/>
+      <c r="C39" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="F39" s="43"/>
+      <c r="G39" s="60"/>
+      <c r="H39" s="60"/>
+      <c r="I39" s="61" t="str">
         <f>IF(AND(G33&lt;&gt;"",H33&lt;&gt;""),H33-G33,"")</f>
         <v/>
       </c>
-      <c r="J39" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K39" s="18" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="40" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="19"/>
-      <c r="C40" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="D40" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E40" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F40" s="23"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="24"/>
-      <c r="I40" s="25" t="str">
+      <c r="J39" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B40" s="17"/>
+      <c r="C40" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="D40" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="F40" s="63"/>
+      <c r="G40" s="64"/>
+      <c r="H40" s="64"/>
+      <c r="I40" s="65" t="str">
         <f>IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34,"")</f>
         <v/>
       </c>
-      <c r="J40" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K40" s="26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="41" spans="2:11" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="31"/>
-      <c r="C41" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="D41" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="E41" s="34" t="s">
-        <v>30</v>
-      </c>
-      <c r="F41" s="35"/>
-      <c r="G41" s="36"/>
-      <c r="H41" s="36"/>
-      <c r="I41" s="37" t="str">
+      <c r="J40" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K40" s="24" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B41" s="9"/>
+      <c r="C41" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F41" s="43"/>
+      <c r="G41" s="60"/>
+      <c r="H41" s="60"/>
+      <c r="I41" s="61" t="str">
         <f>IF(AND(G35&lt;&gt;"",H35&lt;&gt;""),H35-G35,"")</f>
         <v/>
       </c>
-      <c r="J41" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K41" s="38" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="42" spans="2:11" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="19"/>
-      <c r="C42" s="20" t="s">
-        <v>97</v>
-      </c>
-      <c r="D42" s="29" t="s">
+      <c r="J41" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B42" s="17"/>
+      <c r="C42" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="D42" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="E42" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F42" s="23"/>
-      <c r="G42" s="24"/>
-      <c r="H42" s="24"/>
-      <c r="I42" s="25" t="str">
+      <c r="E42" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="F42" s="63"/>
+      <c r="G42" s="64"/>
+      <c r="H42" s="64"/>
+      <c r="I42" s="65" t="str">
         <f>IF(AND(G36&lt;&gt;"",H36&lt;&gt;""),H36-G36,"")</f>
         <v/>
       </c>
-      <c r="J42" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K42" s="26" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="43" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="10"/>
-      <c r="C43" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="D43" s="12" t="s">
+      <c r="J42" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K42" s="24" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B43" s="9"/>
+      <c r="C43" s="89" t="s">
+        <v>210</v>
+      </c>
+      <c r="D43" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="E43" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="F43" s="43"/>
+      <c r="G43" s="60"/>
+      <c r="H43" s="60"/>
+      <c r="I43" s="61"/>
+      <c r="J43" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B44" s="17"/>
+      <c r="C44" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="D44" s="69" t="s">
+        <v>25</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="F44" s="63"/>
+      <c r="G44" s="64"/>
+      <c r="H44" s="64"/>
+      <c r="I44" s="65"/>
+      <c r="J44" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K44" s="24" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B45" s="9"/>
+      <c r="C45" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D45" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="F45" s="43"/>
+      <c r="G45" s="60"/>
+      <c r="H45" s="60"/>
+      <c r="I45" s="61" t="str">
+        <f t="shared" ref="I45:I46" si="3">IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37,"")</f>
+        <v/>
+      </c>
+      <c r="J45" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="92"/>
+      <c r="C46" s="93" t="s">
+        <v>207</v>
+      </c>
+      <c r="D46" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="F43" s="14"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="16" t="str">
-        <f>IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37,"")</f>
+      <c r="E46" s="95" t="s">
+        <v>31</v>
+      </c>
+      <c r="F46" s="96"/>
+      <c r="G46" s="97"/>
+      <c r="H46" s="97"/>
+      <c r="I46" s="98" t="str">
+        <f t="shared" ref="I46" si="4">IF(AND(G46&lt;&gt;"",H46&lt;&gt;""),H46-G46,"")</f>
         <v/>
       </c>
-      <c r="J43" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K43" s="18" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="44" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="19"/>
-      <c r="C44" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="D44" s="29" t="s">
+      <c r="J46" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K46" s="99" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="48" spans="1:11" s="55" customFormat="1" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="56" t="s">
+        <v>146</v>
+      </c>
+      <c r="D48" s="57"/>
+      <c r="E48" s="58" t="s">
+        <v>22</v>
+      </c>
+      <c r="F48" s="57"/>
+      <c r="G48" s="57"/>
+      <c r="H48" s="57"/>
+      <c r="I48" s="57"/>
+      <c r="J48" s="59" t="s">
+        <v>18</v>
+      </c>
+      <c r="K48" s="8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A49"/>
+      <c r="B49" s="9"/>
+      <c r="C49" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D49" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="F49" s="43"/>
+      <c r="G49" s="60"/>
+      <c r="H49" s="60"/>
+      <c r="I49" s="61" t="str">
+        <f t="shared" ref="I49:I56" si="5">IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),H49-G49,"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A50"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="D50" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E50" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="F50" s="63"/>
+      <c r="G50" s="64"/>
+      <c r="H50" s="64"/>
+      <c r="I50" s="65" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J50" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K50" s="24" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A51"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="D51" s="66" t="s">
+        <v>21</v>
+      </c>
+      <c r="E51" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="F51" s="50"/>
+      <c r="G51" s="67"/>
+      <c r="H51" s="67"/>
+      <c r="I51" s="68" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J51" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K51" s="36" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A52"/>
+      <c r="B52" s="17"/>
+      <c r="C52" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="D52" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="E52" s="88" t="s">
+        <v>204</v>
+      </c>
+      <c r="F52" s="63"/>
+      <c r="G52" s="64"/>
+      <c r="H52" s="64"/>
+      <c r="I52" s="65" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J52" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K52" s="24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A53"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D53" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F53" s="43"/>
+      <c r="G53" s="60"/>
+      <c r="H53" s="60"/>
+      <c r="I53" s="61" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J53" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K53" s="86" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A54"/>
+      <c r="B54" s="17"/>
+      <c r="C54" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D54" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="E44" s="22" t="s">
+      <c r="E54" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="F54" s="63"/>
+      <c r="G54" s="64"/>
+      <c r="H54" s="64"/>
+      <c r="I54" s="65" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J54" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K54" s="71" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A55"/>
+      <c r="B55" s="9"/>
+      <c r="C55" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D55" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E55" s="89" t="s">
+        <v>204</v>
+      </c>
+      <c r="F55" s="43"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="61" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J55" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K55" s="87" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" s="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A56"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D56" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="F44" s="23"/>
-      <c r="G44" s="24"/>
-      <c r="H44" s="24"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="K44" s="18" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="45" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="10"/>
-      <c r="C45" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="D45" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F45" s="14"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="16"/>
-      <c r="J45" s="17" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="2:11" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="19"/>
-      <c r="C46" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E46" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F46" s="23"/>
-      <c r="G46" s="24"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="25" t="str">
-        <f t="shared" ref="I46:I48" si="3">IF(AND(G38&lt;&gt;"",H38&lt;&gt;""),H38-G38,"")</f>
+      <c r="E56" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="F56" s="63"/>
+      <c r="G56" s="64"/>
+      <c r="H56" s="64"/>
+      <c r="I56" s="65" t="str">
+        <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J46" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K46" s="26" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="47" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="10"/>
-      <c r="C47" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="D47" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="F47" s="14"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="16" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J47" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K47" s="18" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="48" spans="2:11" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="19"/>
-      <c r="C48" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="D48" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="E48" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="F48" s="23"/>
-      <c r="G48" s="24"/>
-      <c r="H48" s="24"/>
-      <c r="I48" s="25" t="str">
-        <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="J48" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K48" s="26" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="49" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C51" s="40" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="52" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C52" s="41" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C53" s="42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="54" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C54" s="43" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="55" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C55" s="44" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="56" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C56" s="45" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="57" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="J56" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="K56" s="24" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C59" s="37" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="38" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="39" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C62" s="40" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C63" s="41" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C64" s="42" t="s">
+        <v>88</v>
+      </c>
+    </row>
     <row r="65" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3460,6 +3843,14 @@
     <row r="996" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="997" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="998" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="999" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1000" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1001" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1002" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1003" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1004" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1005" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1006" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J3:K3"/>
@@ -3467,13 +3858,13 @@
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="C3:G3"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J7:J10 J13:J19 J22:J30 J44 J33:J40" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" sqref="J7:J10 J13:J19 J22:J30 J43 J34:J39 J32 J46" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Complete,Overdue,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3490,589 +3881,774 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="26" width="8.6640625" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="10" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="80" t="s">
+      <c r="B1" s="82" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+    </row>
+    <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="83" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+    </row>
+    <row r="3" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="43">
+        <v>1</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" s="43"/>
+      <c r="H4" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="10"/>
+    </row>
+    <row r="5" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="45">
+        <v>2</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="45"/>
+      <c r="H5" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="46"/>
+    </row>
+    <row r="6" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="43">
+        <v>3</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6" s="43"/>
+      <c r="H6" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="10"/>
+    </row>
+    <row r="7" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="45">
+        <v>4</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" s="45"/>
+      <c r="H7" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="46"/>
+    </row>
+    <row r="8" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="43">
+        <v>5</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G8" s="43"/>
+      <c r="H8" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="10"/>
+    </row>
+    <row r="9" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="45">
+        <v>6</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" s="45"/>
+      <c r="H9" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="46"/>
+    </row>
+    <row r="10" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="43">
+        <v>7</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="43"/>
+      <c r="H10" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="10"/>
+    </row>
+    <row r="11" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="45">
+        <v>8</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="45"/>
+      <c r="H11" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="46"/>
+    </row>
+    <row r="12" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="43">
+        <v>9</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="43" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-    </row>
-    <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="81" t="s">
+      <c r="E12" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12" s="43"/>
+      <c r="H12" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="10"/>
+    </row>
+    <row r="13" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="45">
+        <v>10</v>
+      </c>
+      <c r="C13" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-    </row>
-    <row r="3" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="3" t="s">
+      <c r="D13" s="45" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E13" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G13" s="45"/>
+      <c r="H13" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" s="46"/>
+    </row>
+    <row r="14" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="43">
+        <v>11</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D14" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E14" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="43"/>
+      <c r="H14" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I14" s="10"/>
+    </row>
+    <row r="15" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="45">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="C15" s="46" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" s="45" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G15" s="45"/>
+      <c r="H15" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="46"/>
+    </row>
+    <row r="16" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="43">
+        <v>13</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" s="43"/>
+      <c r="H16" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="10"/>
+    </row>
+    <row r="17" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="45">
         <v>14</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="46">
-        <v>1</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>122</v>
-      </c>
-      <c r="E4" s="47" t="s">
+      <c r="C17" s="46" t="s">
+        <v>124</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="G17" s="45"/>
+      <c r="H17" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="46"/>
+    </row>
+    <row r="18" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="43">
+        <v>15</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G18" s="43"/>
+      <c r="H18" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I18" s="10"/>
+    </row>
+    <row r="19" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="45">
+        <v>16</v>
+      </c>
+      <c r="C19" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19" s="45" t="s">
+        <v>129</v>
+      </c>
+      <c r="E19" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G4" s="46"/>
-      <c r="H4" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="48">
-        <v>2</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="D5" s="48" t="s">
-        <v>125</v>
-      </c>
-      <c r="E5" s="50" t="s">
+      <c r="F19" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19" s="45"/>
+      <c r="H19" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="46"/>
+    </row>
+    <row r="20" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="43">
+        <v>17</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>131</v>
+      </c>
+      <c r="E20" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="48" t="s">
-        <v>123</v>
-      </c>
-      <c r="G5" s="48"/>
-      <c r="H5" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I5" s="49"/>
-    </row>
-    <row r="6" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="46">
-        <v>3</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="E6" s="47" t="s">
+      <c r="F20" s="43" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" s="43"/>
+      <c r="H20" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="10"/>
+    </row>
+    <row r="21" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="45">
+        <v>18</v>
+      </c>
+      <c r="C21" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="E21" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G6" s="46"/>
-      <c r="H6" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I6" s="11"/>
-    </row>
-    <row r="7" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="48">
-        <v>4</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>128</v>
-      </c>
-      <c r="D7" s="48" t="s">
-        <v>129</v>
-      </c>
-      <c r="E7" s="50" t="s">
+      <c r="F21" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="45"/>
+      <c r="H21" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="46"/>
+    </row>
+    <row r="22" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="50">
+        <v>19</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="D22" s="50" t="s">
+        <v>135</v>
+      </c>
+      <c r="E22" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="50" t="s">
+        <v>164</v>
+      </c>
+      <c r="G22" s="50"/>
+      <c r="H22" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I22" s="30"/>
+    </row>
+    <row r="23" spans="2:9" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="45">
+        <v>20</v>
+      </c>
+      <c r="C23" s="46" t="s">
+        <v>136</v>
+      </c>
+      <c r="D23" s="45" t="s">
+        <v>137</v>
+      </c>
+      <c r="E23" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="48" t="s">
-        <v>123</v>
-      </c>
-      <c r="G7" s="48"/>
-      <c r="H7" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I7" s="49"/>
-    </row>
-    <row r="8" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="46">
-        <v>5</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>131</v>
-      </c>
-      <c r="E8" s="47" t="s">
+      <c r="F23" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G23" s="45"/>
+      <c r="H23" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" s="46"/>
+    </row>
+    <row r="24" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="50">
+        <v>21</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="G24" s="50"/>
+      <c r="H24" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I24" s="30"/>
+    </row>
+    <row r="25" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="52">
+        <v>22</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="52" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="G25" s="52"/>
+      <c r="H25" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I25" s="53" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="52">
+        <v>23</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>144</v>
+      </c>
+      <c r="D26" s="52" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="G26" s="52"/>
+      <c r="H26" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="53" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B27" s="45">
+        <v>24</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="E27" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="45" t="s">
+        <v>164</v>
+      </c>
+      <c r="G27" s="45"/>
+      <c r="H27" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" s="46" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B28" s="43">
         <v>25</v>
       </c>
-      <c r="F8" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G8" s="46"/>
-      <c r="H8" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" s="11"/>
-    </row>
-    <row r="9" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="48">
-        <v>6</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>132</v>
-      </c>
-      <c r="D9" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="E9" s="50" t="s">
+      <c r="C28" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>164</v>
+      </c>
+      <c r="G28" s="43"/>
+      <c r="H28" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B29" s="45">
+        <v>26</v>
+      </c>
+      <c r="C29" s="46" t="s">
+        <v>172</v>
+      </c>
+      <c r="D29" s="45" t="s">
+        <v>173</v>
+      </c>
+      <c r="E29" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G9" s="48"/>
-      <c r="H9" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I9" s="49"/>
-    </row>
-    <row r="10" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="46">
-        <v>7</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="D10" s="46" t="s">
-        <v>136</v>
-      </c>
-      <c r="E10" s="47" t="s">
+      <c r="F29" s="45" t="s">
+        <v>164</v>
+      </c>
+      <c r="G29" s="45"/>
+      <c r="H29" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="46" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B30" s="43">
+        <v>27</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="D30" s="43" t="s">
+        <v>183</v>
+      </c>
+      <c r="E30" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" s="43"/>
+      <c r="H30" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B31" s="45">
+        <v>28</v>
+      </c>
+      <c r="C31" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="D31" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="G31" s="45"/>
+      <c r="H31" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="46" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="B32" s="43">
+        <v>29</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="D32" s="43" t="s">
+        <v>189</v>
+      </c>
+      <c r="E32" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" s="43"/>
+      <c r="H32" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="69" x14ac:dyDescent="0.3">
+      <c r="B33" s="45">
+        <v>30</v>
+      </c>
+      <c r="C33" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="D33" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="E33" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="G33" s="45"/>
+      <c r="H33" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="46" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="B34" s="43">
+        <v>31</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D34" s="43" t="s">
+        <v>195</v>
+      </c>
+      <c r="E34" s="49" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="46" t="s">
-        <v>134</v>
-      </c>
-      <c r="G10" s="46"/>
-      <c r="H10" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I10" s="11"/>
-    </row>
-    <row r="11" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="48">
-        <v>8</v>
-      </c>
-      <c r="C11" s="49" t="s">
-        <v>137</v>
-      </c>
-      <c r="D11" s="48" t="s">
-        <v>138</v>
-      </c>
-      <c r="E11" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G11" s="48"/>
-      <c r="H11" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I11" s="49"/>
-    </row>
-    <row r="12" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="46">
-        <v>9</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="D12" s="46" t="s">
-        <v>140</v>
-      </c>
-      <c r="E12" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="46" t="s">
-        <v>134</v>
-      </c>
-      <c r="G12" s="46"/>
-      <c r="H12" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" s="11"/>
-    </row>
-    <row r="13" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="48">
-        <v>10</v>
-      </c>
-      <c r="C13" s="49" t="s">
-        <v>141</v>
-      </c>
-      <c r="D13" s="48" t="s">
-        <v>142</v>
-      </c>
-      <c r="E13" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G13" s="48"/>
-      <c r="H13" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I13" s="49"/>
-    </row>
-    <row r="14" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="46">
-        <v>11</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="D14" s="46" t="s">
-        <v>144</v>
-      </c>
-      <c r="E14" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="G14" s="46"/>
-      <c r="H14" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I14" s="11"/>
-    </row>
-    <row r="15" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="48">
-        <v>12</v>
-      </c>
-      <c r="C15" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="D15" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="E15" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="48" t="s">
-        <v>145</v>
-      </c>
-      <c r="G15" s="48"/>
-      <c r="H15" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I15" s="49"/>
-    </row>
-    <row r="16" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="46">
-        <v>13</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D16" s="46" t="s">
-        <v>149</v>
-      </c>
-      <c r="E16" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="G16" s="46"/>
-      <c r="H16" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I16" s="11"/>
-    </row>
-    <row r="17" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="48">
-        <v>14</v>
-      </c>
-      <c r="C17" s="49" t="s">
-        <v>150</v>
-      </c>
-      <c r="D17" s="48" t="s">
-        <v>151</v>
-      </c>
-      <c r="E17" s="50" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" s="48" t="s">
-        <v>145</v>
-      </c>
-      <c r="G17" s="48"/>
-      <c r="H17" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I17" s="49"/>
-    </row>
-    <row r="18" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="46">
-        <v>15</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>153</v>
-      </c>
-      <c r="E18" s="47" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" s="46" t="s">
-        <v>145</v>
-      </c>
-      <c r="G18" s="46"/>
-      <c r="H18" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I18" s="11"/>
-    </row>
-    <row r="19" spans="2:9" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="48">
-        <v>16</v>
-      </c>
-      <c r="C19" s="49" t="s">
-        <v>154</v>
-      </c>
-      <c r="D19" s="48" t="s">
-        <v>155</v>
-      </c>
-      <c r="E19" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="48" t="s">
-        <v>123</v>
-      </c>
-      <c r="G19" s="48"/>
-      <c r="H19" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I19" s="49"/>
-    </row>
-    <row r="20" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="46">
-        <v>17</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D20" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="E20" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="46" t="s">
-        <v>123</v>
-      </c>
-      <c r="G20" s="46"/>
-      <c r="H20" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I20" s="11"/>
-    </row>
-    <row r="21" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="48">
-        <v>18</v>
-      </c>
-      <c r="C21" s="49" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" s="48" t="s">
-        <v>159</v>
-      </c>
-      <c r="E21" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="F21" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G21" s="48"/>
-      <c r="H21" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I21" s="49"/>
-    </row>
-    <row r="22" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="53">
-        <v>19</v>
-      </c>
-      <c r="C22" s="32" t="s">
-        <v>160</v>
-      </c>
-      <c r="D22" s="53" t="s">
-        <v>161</v>
-      </c>
-      <c r="E22" s="54" t="s">
-        <v>25</v>
-      </c>
-      <c r="F22" s="53" t="s">
-        <v>145</v>
-      </c>
-      <c r="G22" s="53"/>
-      <c r="H22" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I22" s="32"/>
-    </row>
-    <row r="23" spans="2:9" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="48">
-        <v>20</v>
-      </c>
-      <c r="C23" s="49" t="s">
-        <v>162</v>
-      </c>
-      <c r="D23" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="E23" s="51" t="s">
-        <v>29</v>
-      </c>
-      <c r="F23" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="G23" s="48"/>
-      <c r="H23" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I23" s="49"/>
-    </row>
-    <row r="24" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="53">
-        <v>21</v>
-      </c>
-      <c r="C24" s="32" t="s">
-        <v>164</v>
-      </c>
-      <c r="D24" s="53" t="s">
-        <v>165</v>
-      </c>
-      <c r="E24" s="54" t="s">
-        <v>25</v>
-      </c>
-      <c r="F24" s="53" t="s">
-        <v>145</v>
-      </c>
-      <c r="G24" s="53"/>
-      <c r="H24" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="I24" s="32"/>
-    </row>
-    <row r="25" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="55">
-        <v>22</v>
-      </c>
-      <c r="C25" s="56" t="s">
-        <v>166</v>
-      </c>
-      <c r="D25" s="55" t="s">
-        <v>167</v>
-      </c>
-      <c r="E25" s="55" t="s">
-        <v>25</v>
-      </c>
-      <c r="F25" s="55" t="s">
-        <v>168</v>
-      </c>
-      <c r="G25" s="55"/>
-      <c r="H25" s="57" t="s">
-        <v>89</v>
-      </c>
-      <c r="I25" s="56" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="55">
-        <v>23</v>
-      </c>
-      <c r="C26" s="56" t="s">
-        <v>170</v>
-      </c>
-      <c r="D26" s="55" t="s">
-        <v>171</v>
-      </c>
-      <c r="E26" s="55" t="s">
-        <v>25</v>
-      </c>
-      <c r="F26" s="55" t="s">
-        <v>168</v>
-      </c>
-      <c r="G26" s="55"/>
-      <c r="H26" s="57" t="s">
-        <v>89</v>
-      </c>
-      <c r="I26" s="56" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="F34" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="G34" s="43"/>
+      <c r="H34" s="73" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="49" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="50" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="51" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
bổ sung công việc
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F245A2D4-DACD-4B43-8E31-A644E5D92668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90749CF9-F03C-4D97-A521-7261E859CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="213">
   <si>
     <t>KẾ HOẠCH DỰ ÁN THEO AGILE/SCRUM</t>
   </si>
@@ -672,6 +672,12 @@
   </si>
   <si>
     <t xml:space="preserve">    Cập nhật Audit Log</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Hoàn thiện tài liệu</t>
+  </si>
+  <si>
+    <t>Hoàn thiện tài liệu dự án.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +812,7 @@
       <charset val="163"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -913,6 +919,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1092,7 +1104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1295,9 +1307,6 @@
     <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1306,6 +1315,55 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1329,53 +1387,25 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="18" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1622,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1006"/>
+  <dimension ref="A1:K1007"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" customWidth="1"/>
@@ -1639,24 +1669,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
     </row>
     <row r="2" spans="2:11" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="84" t="s">
+      <c r="D2" s="73" t="s">
         <v>199</v>
       </c>
       <c r="E2" s="1" t="s">
@@ -1665,30 +1695,30 @@
       <c r="F2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="G2" s="85"/>
+      <c r="G2" s="74"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="76" t="s">
+      <c r="J2" s="92" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="77"/>
+      <c r="K2" s="93"/>
     </row>
     <row r="3" spans="2:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="80" t="s">
+      <c r="C3" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="75"/>
+      <c r="D3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="91"/>
       <c r="H3" s="54">
         <v>1</v>
       </c>
-      <c r="J3" s="74" t="s">
+      <c r="J3" s="90" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="75"/>
+      <c r="K3" s="91"/>
     </row>
     <row r="4" spans="2:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1761,7 +1791,7 @@
         <f>IF(AND(G7&lt;&gt;"",H7&lt;&gt;""),H7-G7,"")</f>
         <v/>
       </c>
-      <c r="J7" s="72" t="s">
+      <c r="J7" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K7" s="16" t="s">
@@ -1776,7 +1806,7 @@
       <c r="D8" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="91" t="s">
+      <c r="E8" s="80" t="s">
         <v>31</v>
       </c>
       <c r="F8" s="21"/>
@@ -1786,7 +1816,7 @@
         <f>IF(AND(G8&lt;&gt;"",H8&lt;&gt;""),H8-G8,"")</f>
         <v/>
       </c>
-      <c r="J8" s="72" t="s">
+      <c r="J8" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="24" t="s">
@@ -1811,7 +1841,7 @@
         <f>IF(AND(G9&lt;&gt;"",H9&lt;&gt;""),H9-G9,"")</f>
         <v/>
       </c>
-      <c r="J9" s="72" t="s">
+      <c r="J9" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K9" s="16" t="s">
@@ -1826,7 +1856,7 @@
       <c r="D10" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="91" t="s">
+      <c r="E10" s="80" t="s">
         <v>31</v>
       </c>
       <c r="F10" s="21"/>
@@ -1836,7 +1866,7 @@
         <f>IF(AND(G10&lt;&gt;"",H10&lt;&gt;""),H10-G10,"")</f>
         <v/>
       </c>
-      <c r="J10" s="72" t="s">
+      <c r="J10" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="24" t="s">
@@ -1882,7 +1912,7 @@
         <f t="shared" ref="I13:I19" si="0">IF(AND(G13&lt;&gt;"",H13&lt;&gt;""),H13-G13,"")</f>
         <v/>
       </c>
-      <c r="J13" s="72" t="s">
+      <c r="J13" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="16" t="s">
@@ -1907,7 +1937,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J14" s="72" t="s">
+      <c r="J14" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="24" t="s">
@@ -1932,7 +1962,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J15" s="72" t="s">
+      <c r="J15" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K15" s="16" t="s">
@@ -1957,7 +1987,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J16" s="72" t="s">
+      <c r="J16" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K16" s="24" t="s">
@@ -1982,7 +2012,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J17" s="72" t="s">
+      <c r="J17" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K17" s="16" t="s">
@@ -2007,7 +2037,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J18" s="72" t="s">
+      <c r="J18" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K18" s="24" t="s">
@@ -2032,7 +2062,7 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J19" s="72" t="s">
+      <c r="J19" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K19" s="16" t="s">
@@ -2078,7 +2108,7 @@
         <f t="shared" ref="I22:I32" si="1">IF(AND(G22&lt;&gt;"",H22&lt;&gt;""),H22-G22,"")</f>
         <v/>
       </c>
-      <c r="J22" s="72" t="s">
+      <c r="J22" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K22" s="16" t="s">
@@ -2103,7 +2133,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J23" s="72" t="s">
+      <c r="J23" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K23" s="24" t="s">
@@ -2118,7 +2148,7 @@
       <c r="D24" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="90" t="s">
+      <c r="E24" s="79" t="s">
         <v>205</v>
       </c>
       <c r="F24" s="13"/>
@@ -2128,7 +2158,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J24" s="72" t="s">
+      <c r="J24" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K24" s="16" t="s">
@@ -2137,7 +2167,7 @@
     </row>
     <row r="25" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="17"/>
-      <c r="C25" s="88" t="s">
+      <c r="C25" s="77" t="s">
         <v>57</v>
       </c>
       <c r="D25" s="19" t="s">
@@ -2153,10 +2183,10 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J25" s="72" t="s">
-        <v>18</v>
-      </c>
-      <c r="K25" s="100" t="s">
+      <c r="J25" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="K25" s="89" t="s">
         <v>209</v>
       </c>
     </row>
@@ -2178,7 +2208,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J26" s="72" t="s">
+      <c r="J26" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K26" s="36" t="s">
@@ -2193,7 +2223,7 @@
       <c r="D27" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="91" t="s">
+      <c r="E27" s="80" t="s">
         <v>205</v>
       </c>
       <c r="F27" s="21"/>
@@ -2203,7 +2233,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J27" s="72" t="s">
+      <c r="J27" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K27" s="24" t="s">
@@ -2228,7 +2258,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J28" s="72" t="s">
+      <c r="J28" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K28" s="36" t="s">
@@ -2253,7 +2283,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J29" s="72" t="s">
+      <c r="J29" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K29" s="24" t="s">
@@ -2278,7 +2308,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J30" s="73" t="s">
+      <c r="J30" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K30" s="16" t="s">
@@ -2303,7 +2333,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J31" s="73" t="s">
+      <c r="J31" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K31" s="24" t="s">
@@ -2312,7 +2342,7 @@
     </row>
     <row r="32" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9"/>
-      <c r="C32" s="89" t="s">
+      <c r="C32" s="78" t="s">
         <v>206</v>
       </c>
       <c r="D32" s="28" t="s">
@@ -2328,7 +2358,7 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J32" s="72" t="s">
+      <c r="J32" s="71" t="s">
         <v>18</v>
       </c>
       <c r="K32" s="16" t="s">
@@ -2371,10 +2401,10 @@
       <c r="G35" s="60"/>
       <c r="H35" s="60"/>
       <c r="I35" s="61" t="str">
-        <f t="shared" ref="I32:I36" si="2">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34,"")</f>
+        <f t="shared" ref="I35:I36" si="2">IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34,"")</f>
         <v/>
       </c>
-      <c r="J35" s="73" t="s">
+      <c r="J35" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K35" s="16" t="s">
@@ -2399,7 +2429,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="J36" s="73" t="s">
+      <c r="J36" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K36" s="24" t="s">
@@ -2421,7 +2451,7 @@
       <c r="G37" s="60"/>
       <c r="H37" s="60"/>
       <c r="I37" s="61"/>
-      <c r="J37" s="73" t="s">
+      <c r="J37" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K37" s="16" t="s">
@@ -2446,7 +2476,7 @@
         <f>IF(AND(G32&lt;&gt;"",H32&lt;&gt;""),H32-G32,"")</f>
         <v/>
       </c>
-      <c r="J38" s="73" t="s">
+      <c r="J38" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K38" s="24" t="s">
@@ -2471,7 +2501,7 @@
         <f>IF(AND(G33&lt;&gt;"",H33&lt;&gt;""),H33-G33,"")</f>
         <v/>
       </c>
-      <c r="J39" s="73" t="s">
+      <c r="J39" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K39" s="16" t="s">
@@ -2496,7 +2526,7 @@
         <f>IF(AND(G34&lt;&gt;"",H34&lt;&gt;""),H34-G34,"")</f>
         <v/>
       </c>
-      <c r="J40" s="73" t="s">
+      <c r="J40" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K40" s="24" t="s">
@@ -2521,7 +2551,7 @@
         <f>IF(AND(G35&lt;&gt;"",H35&lt;&gt;""),H35-G35,"")</f>
         <v/>
       </c>
-      <c r="J41" s="73" t="s">
+      <c r="J41" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K41" s="16" t="s">
@@ -2546,7 +2576,7 @@
         <f>IF(AND(G36&lt;&gt;"",H36&lt;&gt;""),H36-G36,"")</f>
         <v/>
       </c>
-      <c r="J42" s="73" t="s">
+      <c r="J42" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K42" s="24" t="s">
@@ -2555,7 +2585,7 @@
     </row>
     <row r="43" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B43" s="9"/>
-      <c r="C43" s="89" t="s">
+      <c r="C43" s="78" t="s">
         <v>210</v>
       </c>
       <c r="D43" s="49" t="s">
@@ -2568,7 +2598,7 @@
       <c r="G43" s="60"/>
       <c r="H43" s="60"/>
       <c r="I43" s="61"/>
-      <c r="J43" s="73" t="s">
+      <c r="J43" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K43" s="16" t="s">
@@ -2584,13 +2614,13 @@
         <v>25</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>202</v>
+        <v>31</v>
       </c>
       <c r="F44" s="63"/>
       <c r="G44" s="64"/>
       <c r="H44" s="64"/>
       <c r="I44" s="65"/>
-      <c r="J44" s="73" t="s">
+      <c r="J44" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K44" s="24" t="s">
@@ -2612,10 +2642,10 @@
       <c r="G45" s="60"/>
       <c r="H45" s="60"/>
       <c r="I45" s="61" t="str">
-        <f t="shared" ref="I45:I46" si="3">IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37,"")</f>
+        <f t="shared" ref="I45" si="3">IF(AND(G37&lt;&gt;"",H37&lt;&gt;""),H37-G37,"")</f>
         <v/>
       </c>
-      <c r="J45" s="73" t="s">
+      <c r="J45" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K45" s="16" t="s">
@@ -2623,27 +2653,27 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="92"/>
-      <c r="C46" s="93" t="s">
+      <c r="B46" s="81"/>
+      <c r="C46" s="82" t="s">
         <v>207</v>
       </c>
-      <c r="D46" s="94" t="s">
+      <c r="D46" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="E46" s="95" t="s">
+      <c r="E46" s="84" t="s">
         <v>31</v>
       </c>
-      <c r="F46" s="96"/>
-      <c r="G46" s="97"/>
-      <c r="H46" s="97"/>
-      <c r="I46" s="98" t="str">
+      <c r="F46" s="85"/>
+      <c r="G46" s="86"/>
+      <c r="H46" s="86"/>
+      <c r="I46" s="87" t="str">
         <f t="shared" ref="I46" si="4">IF(AND(G46&lt;&gt;"",H46&lt;&gt;""),H46-G46,"")</f>
         <v/>
       </c>
-      <c r="J46" s="72" t="s">
-        <v>18</v>
-      </c>
-      <c r="K46" s="99" t="s">
+      <c r="J46" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="K46" s="88" t="s">
         <v>208</v>
       </c>
     </row>
@@ -2685,10 +2715,10 @@
       <c r="G49" s="60"/>
       <c r="H49" s="60"/>
       <c r="I49" s="61" t="str">
-        <f t="shared" ref="I49:I56" si="5">IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),H49-G49,"")</f>
+        <f t="shared" ref="I49:I57" si="5">IF(AND(G49&lt;&gt;"",H49&lt;&gt;""),H49-G49,"")</f>
         <v/>
       </c>
-      <c r="J49" s="73" t="s">
+      <c r="J49" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K49" s="16" t="s">
@@ -2714,7 +2744,7 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J50" s="73" t="s">
+      <c r="J50" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K50" s="24" t="s">
@@ -2740,7 +2770,7 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J51" s="73" t="s">
+      <c r="J51" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K51" s="36" t="s">
@@ -2756,7 +2786,7 @@
       <c r="D52" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="E52" s="88" t="s">
+      <c r="E52" s="77" t="s">
         <v>204</v>
       </c>
       <c r="F52" s="63"/>
@@ -2766,7 +2796,7 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J52" s="73" t="s">
+      <c r="J52" s="72" t="s">
         <v>18</v>
       </c>
       <c r="K52" s="24" t="s">
@@ -2792,10 +2822,10 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J53" s="73" t="s">
-        <v>18</v>
-      </c>
-      <c r="K53" s="86" t="s">
+      <c r="J53" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K53" s="75" t="s">
         <v>157</v>
       </c>
     </row>
@@ -2818,10 +2848,10 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J54" s="73" t="s">
-        <v>18</v>
-      </c>
-      <c r="K54" s="71" t="s">
+      <c r="J54" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K54" s="70" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2834,7 +2864,7 @@
       <c r="D55" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="E55" s="89" t="s">
+      <c r="E55" s="78" t="s">
         <v>204</v>
       </c>
       <c r="F55" s="43"/>
@@ -2844,10 +2874,10 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J55" s="73" t="s">
-        <v>18</v>
-      </c>
-      <c r="K55" s="87" t="s">
+      <c r="J55" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K55" s="76" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2855,10 +2885,10 @@
       <c r="A56"/>
       <c r="B56" s="17"/>
       <c r="C56" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="D56" s="70" t="s">
-        <v>30</v>
+        <v>211</v>
+      </c>
+      <c r="D56" s="69" t="s">
+        <v>25</v>
       </c>
       <c r="E56" s="18" t="s">
         <v>31</v>
@@ -2867,64 +2897,89 @@
       <c r="G56" s="64"/>
       <c r="H56" s="64"/>
       <c r="I56" s="65" t="str">
+        <f>IF(AND(G56&lt;&gt;"",H56&lt;&gt;""),H56-G56,"")</f>
+        <v/>
+      </c>
+      <c r="J56" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K56" s="70" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" s="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A57"/>
+      <c r="B57" s="100"/>
+      <c r="C57" s="101" t="s">
+        <v>162</v>
+      </c>
+      <c r="D57" s="102" t="s">
+        <v>30</v>
+      </c>
+      <c r="E57" s="101" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" s="103"/>
+      <c r="G57" s="104"/>
+      <c r="H57" s="104"/>
+      <c r="I57" s="105" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J56" s="73" t="s">
-        <v>18</v>
-      </c>
-      <c r="K56" s="24" t="s">
+      <c r="J57" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="K57" s="106" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C59" s="37" t="s">
+    <row r="59" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="37" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C60" s="38" t="s">
+    <row r="61" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="38" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C61" s="39" t="s">
+    <row r="62" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C62" s="39" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C62" s="40" t="s">
-        <v>18</v>
-      </c>
-    </row>
     <row r="63" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C63" s="41" t="s">
+      <c r="C63" s="40" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C64" s="41" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C64" s="42" t="s">
+    <row r="65" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="42" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="65" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="66" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="67" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="68" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="69" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="70" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="71" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="72" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="73" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="74" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="75" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="76" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="77" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="78" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="79" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="80" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="66" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="67" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="68" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="70" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="72" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="73" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="74" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="75" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="76" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="80" spans="3:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="81" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="82" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="83" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3851,6 +3906,7 @@
     <row r="1004" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1005" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="1006" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1007" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J3:K3"/>
@@ -3886,26 +3942,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="82" t="s">
+      <c r="B1" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="83" t="s">
+      <c r="B2" s="99" t="s">
         <v>165</v>
       </c>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
     </row>
     <row r="3" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
@@ -3950,7 +4006,7 @@
         <v>97</v>
       </c>
       <c r="G4" s="43"/>
-      <c r="H4" s="73" t="s">
+      <c r="H4" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="10"/>
@@ -3972,7 +4028,7 @@
         <v>97</v>
       </c>
       <c r="G5" s="45"/>
-      <c r="H5" s="73" t="s">
+      <c r="H5" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I5" s="46"/>
@@ -3994,7 +4050,7 @@
         <v>97</v>
       </c>
       <c r="G6" s="43"/>
-      <c r="H6" s="73" t="s">
+      <c r="H6" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="10"/>
@@ -4016,7 +4072,7 @@
         <v>97</v>
       </c>
       <c r="G7" s="45"/>
-      <c r="H7" s="73" t="s">
+      <c r="H7" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I7" s="46"/>
@@ -4038,7 +4094,7 @@
         <v>97</v>
       </c>
       <c r="G8" s="43"/>
-      <c r="H8" s="73" t="s">
+      <c r="H8" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I8" s="10"/>
@@ -4060,7 +4116,7 @@
         <v>108</v>
       </c>
       <c r="G9" s="45"/>
-      <c r="H9" s="73" t="s">
+      <c r="H9" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I9" s="46"/>
@@ -4082,7 +4138,7 @@
         <v>108</v>
       </c>
       <c r="G10" s="43"/>
-      <c r="H10" s="73" t="s">
+      <c r="H10" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I10" s="10"/>
@@ -4104,7 +4160,7 @@
         <v>108</v>
       </c>
       <c r="G11" s="45"/>
-      <c r="H11" s="73" t="s">
+      <c r="H11" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I11" s="46"/>
@@ -4126,7 +4182,7 @@
         <v>108</v>
       </c>
       <c r="G12" s="43"/>
-      <c r="H12" s="73" t="s">
+      <c r="H12" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I12" s="10"/>
@@ -4148,7 +4204,7 @@
         <v>108</v>
       </c>
       <c r="G13" s="45"/>
-      <c r="H13" s="73" t="s">
+      <c r="H13" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I13" s="46"/>
@@ -4170,7 +4226,7 @@
         <v>119</v>
       </c>
       <c r="G14" s="43"/>
-      <c r="H14" s="73" t="s">
+      <c r="H14" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I14" s="10"/>
@@ -4192,7 +4248,7 @@
         <v>119</v>
       </c>
       <c r="G15" s="45"/>
-      <c r="H15" s="73" t="s">
+      <c r="H15" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I15" s="46"/>
@@ -4214,7 +4270,7 @@
         <v>119</v>
       </c>
       <c r="G16" s="43"/>
-      <c r="H16" s="73" t="s">
+      <c r="H16" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I16" s="10"/>
@@ -4236,7 +4292,7 @@
         <v>119</v>
       </c>
       <c r="G17" s="45"/>
-      <c r="H17" s="73" t="s">
+      <c r="H17" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I17" s="46"/>
@@ -4258,7 +4314,7 @@
         <v>119</v>
       </c>
       <c r="G18" s="43"/>
-      <c r="H18" s="73" t="s">
+      <c r="H18" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I18" s="10"/>
@@ -4280,7 +4336,7 @@
         <v>97</v>
       </c>
       <c r="G19" s="45"/>
-      <c r="H19" s="73" t="s">
+      <c r="H19" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I19" s="46"/>
@@ -4302,7 +4358,7 @@
         <v>97</v>
       </c>
       <c r="G20" s="43"/>
-      <c r="H20" s="73" t="s">
+      <c r="H20" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I20" s="10"/>
@@ -4324,7 +4380,7 @@
         <v>108</v>
       </c>
       <c r="G21" s="45"/>
-      <c r="H21" s="73" t="s">
+      <c r="H21" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I21" s="46"/>
@@ -4346,7 +4402,7 @@
         <v>164</v>
       </c>
       <c r="G22" s="50"/>
-      <c r="H22" s="73" t="s">
+      <c r="H22" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I22" s="30"/>
@@ -4368,7 +4424,7 @@
         <v>108</v>
       </c>
       <c r="G23" s="45"/>
-      <c r="H23" s="73" t="s">
+      <c r="H23" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I23" s="46"/>
@@ -4390,7 +4446,7 @@
         <v>119</v>
       </c>
       <c r="G24" s="50"/>
-      <c r="H24" s="73" t="s">
+      <c r="H24" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I24" s="30"/>
@@ -4412,7 +4468,7 @@
         <v>164</v>
       </c>
       <c r="G25" s="52"/>
-      <c r="H25" s="73" t="s">
+      <c r="H25" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I25" s="53" t="s">
@@ -4436,7 +4492,7 @@
         <v>164</v>
       </c>
       <c r="G26" s="52"/>
-      <c r="H26" s="73" t="s">
+      <c r="H26" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I26" s="53" t="s">
@@ -4460,7 +4516,7 @@
         <v>164</v>
       </c>
       <c r="G27" s="45"/>
-      <c r="H27" s="73" t="s">
+      <c r="H27" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I27" s="46" t="s">
@@ -4484,7 +4540,7 @@
         <v>164</v>
       </c>
       <c r="G28" s="43"/>
-      <c r="H28" s="73" t="s">
+      <c r="H28" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I28" s="10" t="s">
@@ -4508,7 +4564,7 @@
         <v>164</v>
       </c>
       <c r="G29" s="45"/>
-      <c r="H29" s="73" t="s">
+      <c r="H29" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I29" s="46" t="s">
@@ -4532,7 +4588,7 @@
         <v>108</v>
       </c>
       <c r="G30" s="43"/>
-      <c r="H30" s="73" t="s">
+      <c r="H30" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I30" s="10" t="s">
@@ -4556,7 +4612,7 @@
         <v>108</v>
       </c>
       <c r="G31" s="45"/>
-      <c r="H31" s="73" t="s">
+      <c r="H31" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I31" s="46" t="s">
@@ -4580,7 +4636,7 @@
         <v>108</v>
       </c>
       <c r="G32" s="43"/>
-      <c r="H32" s="73" t="s">
+      <c r="H32" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I32" s="10" t="s">
@@ -4604,7 +4660,7 @@
         <v>119</v>
       </c>
       <c r="G33" s="45"/>
-      <c r="H33" s="73" t="s">
+      <c r="H33" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I33" s="46" t="s">
@@ -4628,7 +4684,7 @@
         <v>119</v>
       </c>
       <c r="G34" s="43"/>
-      <c r="H34" s="73" t="s">
+      <c r="H34" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I34" s="10" t="s">

</xml_diff>

<commit_message>
cập nhật readme và gộp migration
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90749CF9-F03C-4D97-A521-7261E859CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30EAE175-2EA2-4C31-B0E6-5002591A1F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -630,12 +630,6 @@
     <t>bluemoon_schema.sql + migration_v2..v6</t>
   </si>
   <si>
-    <t xml:space="preserve">    Xây dựng hệ thống Database Migration theo phiên bản</t>
-  </si>
-  <si>
-    <t>Migration file đánh số phiên bản: bluemoon_schema.sql + migration_v2</t>
-  </si>
-  <si>
     <t>TEAM LEADER: Lê Quang Huy
 PRODUCT OWNER: Lê Quang Huy
 SCRUM MASTER: Trần Khánh Linh</t>
@@ -678,6 +672,12 @@
   </si>
   <si>
     <t>Hoàn thiện tài liệu dự án.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Bổ sung hệ thống Database Migration vào schema</t>
+  </si>
+  <si>
+    <t>Thêm vào bluemoon_schema.sql các migration cho các bản mở rộng</t>
   </si>
 </sst>
 </file>
@@ -1365,6 +1365,27 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1386,27 +1407,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="19" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="19" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1669,56 +1669,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="94" t="s">
+      <c r="B1" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
+      <c r="I1" s="102"/>
+      <c r="J1" s="102"/>
+      <c r="K1" s="102"/>
     </row>
     <row r="2" spans="2:11" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="73" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="F2" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G2" s="74"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="92" t="s">
+      <c r="J2" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="93"/>
+      <c r="K2" s="100"/>
     </row>
     <row r="3" spans="2:11" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="96" t="s">
+      <c r="C3" s="103" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="97"/>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="91"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="98"/>
       <c r="H3" s="54">
         <v>1</v>
       </c>
-      <c r="J3" s="90" t="s">
+      <c r="J3" s="97" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="91"/>
+      <c r="K3" s="98"/>
     </row>
     <row r="4" spans="2:11" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1903,7 +1903,7 @@
         <v>21</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="14"/>
@@ -1928,7 +1928,7 @@
         <v>21</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="22"/>
@@ -1953,7 +1953,7 @@
         <v>21</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="14"/>
@@ -1978,7 +1978,7 @@
         <v>21</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
@@ -2003,7 +2003,7 @@
         <v>21</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="14"/>
@@ -2028,7 +2028,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F18" s="21"/>
       <c r="G18" s="22"/>
@@ -2099,7 +2099,7 @@
         <v>21</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="14"/>
@@ -2124,7 +2124,7 @@
         <v>21</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
@@ -2149,7 +2149,7 @@
         <v>21</v>
       </c>
       <c r="E24" s="79" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="14"/>
@@ -2174,7 +2174,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="22"/>
@@ -2187,7 +2187,7 @@
         <v>18</v>
       </c>
       <c r="K25" s="89" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2199,7 +2199,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F26" s="33"/>
       <c r="G26" s="34"/>
@@ -2224,7 +2224,7 @@
         <v>21</v>
       </c>
       <c r="E27" s="80" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F27" s="21"/>
       <c r="G27" s="22"/>
@@ -2249,7 +2249,7 @@
         <v>21</v>
       </c>
       <c r="E28" s="32" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F28" s="33"/>
       <c r="G28" s="34"/>
@@ -2274,7 +2274,7 @@
         <v>25</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="22"/>
@@ -2299,7 +2299,7 @@
         <v>21</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F30" s="43"/>
       <c r="G30" s="60"/>
@@ -2324,7 +2324,7 @@
         <v>21</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F31" s="63"/>
       <c r="G31" s="64"/>
@@ -2343,7 +2343,7 @@
     <row r="32" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9"/>
       <c r="C32" s="78" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D32" s="28" t="s">
         <v>30</v>
@@ -2395,7 +2395,7 @@
         <v>21</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F35" s="43"/>
       <c r="G35" s="60"/>
@@ -2420,7 +2420,7 @@
         <v>21</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F36" s="63"/>
       <c r="G36" s="64"/>
@@ -2445,7 +2445,7 @@
         <v>21</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F37" s="43"/>
       <c r="G37" s="60"/>
@@ -2467,7 +2467,7 @@
         <v>21</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F38" s="63"/>
       <c r="G38" s="64"/>
@@ -2492,7 +2492,7 @@
         <v>21</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F39" s="43"/>
       <c r="G39" s="60"/>
@@ -2517,7 +2517,7 @@
         <v>21</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F40" s="63"/>
       <c r="G40" s="64"/>
@@ -2542,7 +2542,7 @@
         <v>21</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F41" s="43"/>
       <c r="G41" s="60"/>
@@ -2561,13 +2561,13 @@
     <row r="42" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B42" s="17"/>
       <c r="C42" s="18" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="D42" s="69" t="s">
         <v>25</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F42" s="63"/>
       <c r="G42" s="64"/>
@@ -2580,19 +2580,19 @@
         <v>18</v>
       </c>
       <c r="K42" s="24" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B43" s="9"/>
       <c r="C43" s="78" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D43" s="49" t="s">
         <v>25</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F43" s="43"/>
       <c r="G43" s="60"/>
@@ -2636,7 +2636,7 @@
         <v>25</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F45" s="43"/>
       <c r="G45" s="60"/>
@@ -2655,7 +2655,7 @@
     <row r="46" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="81"/>
       <c r="C46" s="82" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D46" s="83" t="s">
         <v>30</v>
@@ -2674,7 +2674,7 @@
         <v>18</v>
       </c>
       <c r="K46" s="88" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2709,7 +2709,7 @@
         <v>21</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F49" s="43"/>
       <c r="G49" s="60"/>
@@ -2735,7 +2735,7 @@
         <v>21</v>
       </c>
       <c r="E50" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F50" s="63"/>
       <c r="G50" s="64"/>
@@ -2761,7 +2761,7 @@
         <v>21</v>
       </c>
       <c r="E51" s="30" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F51" s="50"/>
       <c r="G51" s="67"/>
@@ -2787,7 +2787,7 @@
         <v>21</v>
       </c>
       <c r="E52" s="77" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F52" s="63"/>
       <c r="G52" s="64"/>
@@ -2813,7 +2813,7 @@
         <v>21</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F53" s="43"/>
       <c r="G53" s="60"/>
@@ -2839,7 +2839,7 @@
         <v>25</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F54" s="63"/>
       <c r="G54" s="64"/>
@@ -2865,7 +2865,7 @@
         <v>21</v>
       </c>
       <c r="E55" s="78" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F55" s="43"/>
       <c r="G55" s="60"/>
@@ -2885,7 +2885,7 @@
       <c r="A56"/>
       <c r="B56" s="17"/>
       <c r="C56" s="18" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D56" s="69" t="s">
         <v>25</v>
@@ -2904,32 +2904,32 @@
         <v>18</v>
       </c>
       <c r="K56" s="70" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="57" spans="1:11" s="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A57"/>
-      <c r="B57" s="100"/>
-      <c r="C57" s="101" t="s">
+      <c r="B57" s="90"/>
+      <c r="C57" s="91" t="s">
         <v>162</v>
       </c>
-      <c r="D57" s="102" t="s">
+      <c r="D57" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="E57" s="101" t="s">
+      <c r="E57" s="91" t="s">
         <v>31</v>
       </c>
-      <c r="F57" s="103"/>
-      <c r="G57" s="104"/>
-      <c r="H57" s="104"/>
-      <c r="I57" s="105" t="str">
+      <c r="F57" s="93"/>
+      <c r="G57" s="94"/>
+      <c r="H57" s="94"/>
+      <c r="I57" s="95" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="J57" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="K57" s="106" t="s">
+      <c r="K57" s="96" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3942,26 +3942,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="98" t="s">
+      <c r="B1" s="105" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="99" t="s">
+      <c r="B2" s="106" t="s">
         <v>165</v>
       </c>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
     </row>
     <row r="3" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
sửa lại file kế hoạch
</commit_message>
<xml_diff>
--- a/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
+++ b/docs/Nhóm 16/01 - Tai lieu du an/2. Ke hoach du an phan mem/KeHoach_Scrum_BlueMoon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BlueMoon\docs\Nhóm 16\01 - Tai lieu du an\2. Ke hoach du an phan mem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30EAE175-2EA2-4C31-B0E6-5002591A1F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0983C7CC-BB1B-4460-826D-31C6F2EEAAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kế hoạch dự án" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="214">
   <si>
     <t>KẾ HOẠCH DỰ ÁN THEO AGILE/SCRUM</t>
   </si>
@@ -480,9 +480,6 @@
     <t>Sprint 4 — v2.0: Phí gửi xe &amp; Thu hộ</t>
   </si>
   <si>
-    <t>Hoàn thiện các tính năng v2.0: quản lý phí gửi xe (PER_XE), thu hộ điện/nước/internet (THU_HO), email nhắc nợ tự động (RL-016, RL-019, RL-020).</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Cài đặt Quản lý phương tiện (PhuongTien CRUD)</t>
   </si>
   <si>
@@ -498,9 +495,6 @@
     <t xml:space="preserve">    Cài đặt loại phí THU_HO (thu hộ điện/nước/internet)</t>
   </si>
   <si>
-    <t>Nhập số tiền riêng từng hộ qua form nhap-thu-ho. Liên kết RL-020.</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Cài đặt Mẫu khoản thu định kỳ (MauKhoanThu)</t>
   </si>
   <si>
@@ -579,9 +573,6 @@
     <t>Bảng tất cả hộ vs trạng thái đóng phí tại /thanh-toan/theo-doi dùng paymentMap.</t>
   </si>
   <si>
-    <t>Ghi log theo format [AUDIT] Tạo|Sửa|Xóa entity bằng @Slf4j thay vì bảng DB riêng. Liên kết RL-023.</t>
-  </si>
-  <si>
     <t>Tuân thủ Java Coding Convention, Javadocs.</t>
   </si>
   <si>
@@ -625,9 +616,6 @@
   </si>
   <si>
     <t>Hệ thống phải hỗ trợ migration cơ sở dữ liệu theo phiên bản.</t>
-  </si>
-  <si>
-    <t>bluemoon_schema.sql + migration_v2..v6</t>
   </si>
   <si>
     <t>TEAM LEADER: Lê Quang Huy
@@ -662,9 +650,6 @@
     <t>Demo toàn bộ v1.0, cập nhật Backlog. Lên kế hoạch cho v2.0</t>
   </si>
   <si>
-    <t>Ghi log bằng @Slf4j format [AUDIT] thay vì bảng DB cho các tính năng đã hoàn thành. Liên kết RL-023, NFR-003.</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Cập nhật Audit Log</t>
   </si>
   <si>
@@ -677,7 +662,25 @@
     <t xml:space="preserve">    Bổ sung hệ thống Database Migration vào schema</t>
   </si>
   <si>
-    <t>Thêm vào bluemoon_schema.sql các migration cho các bản mở rộng</t>
+    <t>Quản lý hóa đơn thu hộ điện/nước/internet/gas qua entity HoaDonThuHo tại /thu-ho. Liên kết RL-020.</t>
+  </si>
+  <si>
+    <t>Hoàn thiện các tính năng v2.0: quản lý phí gửi xe (PER_XE), thu hộ điện/nước/internet/gas (HoaDonThuHo), email nhắc nợ tự động (RL-016, RL-019, RL-020).</t>
+  </si>
+  <si>
+    <t>SLF4J log Sprint 2–3; nâng lên bảng audit_log tại Sprint 4</t>
+  </si>
+  <si>
+    <t>Ghi log bằng @Slf4j format [AUDIT] cho v1.0. Nâng cấp lên bảng audit_log ở v2.0. Liên kết RL-023, NFR-003.</t>
+  </si>
+  <si>
+    <t>Ghi log theo format [AUDIT] Tạo|Sửa|Xóa entity bằng @Slf4j. Sẽ nâng lên bảng DB ở v2.0. Liên kết RL-023.</t>
+  </si>
+  <si>
+    <t>Gộp toàn bộ migration vào bluemoon_schema.sql (không dùng file migration riêng).</t>
+  </si>
+  <si>
+    <t>Toàn bộ schema và migration gộp vào bluemoon_schema.sql</t>
   </si>
 </sst>
 </file>
@@ -1630,7 +1633,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="0">
+  <wetp:taskpane dockstate="right" visibility="0" width="455" row="0">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1687,13 +1690,13 @@
         <v>1</v>
       </c>
       <c r="D2" s="73" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="G2" s="74"/>
       <c r="H2" s="1" t="s">
@@ -1903,7 +1906,7 @@
         <v>21</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="14"/>
@@ -1928,7 +1931,7 @@
         <v>21</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="22"/>
@@ -1953,7 +1956,7 @@
         <v>21</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="14"/>
@@ -1978,7 +1981,7 @@
         <v>21</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="22"/>
@@ -2003,7 +2006,7 @@
         <v>21</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="14"/>
@@ -2028,7 +2031,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F18" s="21"/>
       <c r="G18" s="22"/>
@@ -2099,7 +2102,7 @@
         <v>21</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="14"/>
@@ -2124,7 +2127,7 @@
         <v>21</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="22"/>
@@ -2149,7 +2152,7 @@
         <v>21</v>
       </c>
       <c r="E24" s="79" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="14"/>
@@ -2174,7 +2177,7 @@
         <v>25</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="22"/>
@@ -2187,7 +2190,7 @@
         <v>18</v>
       </c>
       <c r="K25" s="89" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2199,7 +2202,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="32" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F26" s="33"/>
       <c r="G26" s="34"/>
@@ -2224,7 +2227,7 @@
         <v>21</v>
       </c>
       <c r="E27" s="80" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F27" s="21"/>
       <c r="G27" s="22"/>
@@ -2249,7 +2252,7 @@
         <v>21</v>
       </c>
       <c r="E28" s="32" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F28" s="33"/>
       <c r="G28" s="34"/>
@@ -2274,7 +2277,7 @@
         <v>25</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="22"/>
@@ -2299,7 +2302,7 @@
         <v>21</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F30" s="43"/>
       <c r="G30" s="60"/>
@@ -2312,7 +2315,7 @@
         <v>18</v>
       </c>
       <c r="K30" s="16" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="2:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -2324,7 +2327,7 @@
         <v>21</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F31" s="63"/>
       <c r="G31" s="64"/>
@@ -2337,13 +2340,13 @@
         <v>18</v>
       </c>
       <c r="K31" s="24" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="9"/>
       <c r="C32" s="78" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D32" s="28" t="s">
         <v>30</v>
@@ -2395,7 +2398,7 @@
         <v>21</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F35" s="43"/>
       <c r="G35" s="60"/>
@@ -2420,7 +2423,7 @@
         <v>21</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F36" s="63"/>
       <c r="G36" s="64"/>
@@ -2445,7 +2448,7 @@
         <v>21</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F37" s="43"/>
       <c r="G37" s="60"/>
@@ -2467,7 +2470,7 @@
         <v>21</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F38" s="63"/>
       <c r="G38" s="64"/>
@@ -2480,7 +2483,7 @@
         <v>18</v>
       </c>
       <c r="K38" s="24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -2492,7 +2495,7 @@
         <v>21</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F39" s="43"/>
       <c r="G39" s="60"/>
@@ -2517,7 +2520,7 @@
         <v>21</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F40" s="63"/>
       <c r="G40" s="64"/>
@@ -2530,7 +2533,7 @@
         <v>18</v>
       </c>
       <c r="K40" s="24" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -2542,7 +2545,7 @@
         <v>21</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F41" s="43"/>
       <c r="G41" s="60"/>
@@ -2555,19 +2558,19 @@
         <v>18</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B42" s="17"/>
       <c r="C42" s="18" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D42" s="69" t="s">
         <v>25</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F42" s="63"/>
       <c r="G42" s="64"/>
@@ -2586,13 +2589,13 @@
     <row r="43" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="B43" s="9"/>
       <c r="C43" s="78" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D43" s="49" t="s">
         <v>25</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F43" s="43"/>
       <c r="G43" s="60"/>
@@ -2602,7 +2605,7 @@
         <v>18</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -2624,7 +2627,7 @@
         <v>18</v>
       </c>
       <c r="K44" s="24" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
@@ -2636,7 +2639,7 @@
         <v>25</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F45" s="43"/>
       <c r="G45" s="60"/>
@@ -2655,7 +2658,7 @@
     <row r="46" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="81"/>
       <c r="C46" s="82" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D46" s="83" t="s">
         <v>30</v>
@@ -2674,7 +2677,7 @@
         <v>18</v>
       </c>
       <c r="K46" s="88" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -2696,20 +2699,20 @@
         <v>18</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>147</v>
+        <v>208</v>
       </c>
     </row>
     <row r="49" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A49"/>
       <c r="B49" s="9"/>
       <c r="C49" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D49" s="44" t="s">
         <v>21</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F49" s="43"/>
       <c r="G49" s="60"/>
@@ -2722,20 +2725,20 @@
         <v>18</v>
       </c>
       <c r="K49" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A50"/>
       <c r="B50" s="17"/>
       <c r="C50" s="18" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D50" s="62" t="s">
         <v>21</v>
       </c>
       <c r="E50" s="18" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F50" s="63"/>
       <c r="G50" s="64"/>
@@ -2748,20 +2751,20 @@
         <v>18</v>
       </c>
       <c r="K50" s="24" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A51"/>
       <c r="B51" s="29"/>
       <c r="C51" s="30" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D51" s="66" t="s">
         <v>21</v>
       </c>
       <c r="E51" s="30" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F51" s="50"/>
       <c r="G51" s="67"/>
@@ -2774,20 +2777,20 @@
         <v>18</v>
       </c>
       <c r="K51" s="36" t="s">
-        <v>153</v>
+        <v>207</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A52"/>
       <c r="B52" s="17"/>
       <c r="C52" s="18" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D52" s="62" t="s">
         <v>21</v>
       </c>
       <c r="E52" s="77" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F52" s="63"/>
       <c r="G52" s="64"/>
@@ -2800,20 +2803,20 @@
         <v>18</v>
       </c>
       <c r="K52" s="24" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A53"/>
       <c r="B53" s="9"/>
       <c r="C53" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D53" s="44" t="s">
         <v>21</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F53" s="43"/>
       <c r="G53" s="60"/>
@@ -2826,20 +2829,20 @@
         <v>18</v>
       </c>
       <c r="K53" s="75" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A54"/>
       <c r="B54" s="17"/>
       <c r="C54" s="18" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D54" s="69" t="s">
         <v>25</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F54" s="63"/>
       <c r="G54" s="64"/>
@@ -2852,20 +2855,20 @@
         <v>18</v>
       </c>
       <c r="K54" s="70" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:11" s="55" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A55"/>
       <c r="B55" s="9"/>
       <c r="C55" s="10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D55" s="44" t="s">
         <v>21</v>
       </c>
       <c r="E55" s="78" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F55" s="43"/>
       <c r="G55" s="60"/>
@@ -2878,14 +2881,14 @@
         <v>18</v>
       </c>
       <c r="K55" s="76" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:11" s="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A56"/>
       <c r="B56" s="17"/>
       <c r="C56" s="18" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D56" s="69" t="s">
         <v>25</v>
@@ -2904,14 +2907,14 @@
         <v>18</v>
       </c>
       <c r="K56" s="70" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="57" spans="1:11" s="55" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A57"/>
       <c r="B57" s="90"/>
       <c r="C57" s="91" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D57" s="92" t="s">
         <v>30</v>
@@ -2930,7 +2933,7 @@
         <v>18</v>
       </c>
       <c r="K57" s="96" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3937,7 +3940,7 @@
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" customWidth="1"/>
     <col min="10" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3954,7 +3957,7 @@
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="106" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C2" s="102"/>
       <c r="D2" s="102"/>
@@ -4399,7 +4402,7 @@
         <v>21</v>
       </c>
       <c r="F22" s="50" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G22" s="50"/>
       <c r="H22" s="72" t="s">
@@ -4427,7 +4430,9 @@
       <c r="H23" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="46"/>
+      <c r="I23" s="46" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="24" spans="2:9" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="50">
@@ -4465,7 +4470,7 @@
         <v>21</v>
       </c>
       <c r="F25" s="52" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G25" s="52"/>
       <c r="H25" s="72" t="s">
@@ -4489,7 +4494,7 @@
         <v>21</v>
       </c>
       <c r="F26" s="52" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G26" s="52"/>
       <c r="H26" s="72" t="s">
@@ -4504,23 +4509,23 @@
         <v>24</v>
       </c>
       <c r="C27" s="46" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E27" s="47" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="45" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G27" s="45"/>
       <c r="H27" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I27" s="46" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
@@ -4528,23 +4533,23 @@
         <v>25</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D28" s="43" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E28" s="44" t="s">
         <v>21</v>
       </c>
       <c r="F28" s="43" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G28" s="43"/>
       <c r="H28" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
@@ -4552,23 +4557,23 @@
         <v>26</v>
       </c>
       <c r="C29" s="46" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D29" s="45" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E29" s="48" t="s">
         <v>25</v>
       </c>
       <c r="F29" s="45" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="G29" s="45"/>
       <c r="H29" s="72" t="s">
         <v>18</v>
       </c>
       <c r="I29" s="46" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
@@ -4576,10 +4581,10 @@
         <v>27</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D30" s="43" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E30" s="44" t="s">
         <v>21</v>
@@ -4592,7 +4597,7 @@
         <v>18</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
@@ -4600,10 +4605,10 @@
         <v>28</v>
       </c>
       <c r="C31" s="46" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D31" s="45" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E31" s="47" t="s">
         <v>21</v>
@@ -4616,7 +4621,7 @@
         <v>18</v>
       </c>
       <c r="I31" s="46" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="2:9" ht="69" x14ac:dyDescent="0.3">
@@ -4624,10 +4629,10 @@
         <v>29</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D32" s="43" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E32" s="44" t="s">
         <v>21</v>
@@ -4640,7 +4645,7 @@
         <v>18</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="69" x14ac:dyDescent="0.3">
@@ -4648,10 +4653,10 @@
         <v>30</v>
       </c>
       <c r="C33" s="46" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D33" s="45" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E33" s="47" t="s">
         <v>21</v>
@@ -4664,7 +4669,7 @@
         <v>18</v>
       </c>
       <c r="I33" s="46" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="2:9" ht="55.2" x14ac:dyDescent="0.3">
@@ -4672,10 +4677,10 @@
         <v>31</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D34" s="43" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E34" s="49" t="s">
         <v>25</v>
@@ -4688,7 +4693,7 @@
         <v>18</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>